<commit_message>
updating several files with fixes for flags
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/Erie/D100/ER 10 D100 Spring 2024 24GE00I73 Zoop.xlsx
+++ b/data/raw/GLNPO 2024 Spring/Erie/D100/ER 10 D100 Spring 2024 24GE00I73 Zoop.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gl Lab User\Box\GLNPO Zooplankton Data\GLNPO 2024 Spring\Erie\D100\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\Erie\D100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9E6CD01-2DD0-4D60-AEDB-0A6713138105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7799DF54-DF35-4256-9F4D-2BD4CFAD0DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{80FB5747-2496-44F2-ACA5-DE03CA5C5388}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80FB5747-2496-44F2-ACA5-DE03CA5C5388}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4830" r:id="rId2"/>
+    <pivotCache cacheId="2" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -4146,7 +4146,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{75DDA9CE-6863-4D74-9189-5E1074C0BE29}" name="PivotTable1" cacheId="4830" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{75DDA9CE-6863-4D74-9189-5E1074C0BE29}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="T2:Y17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
@@ -4594,18 +4594,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A2BCB1-26C9-4765-B0C9-78158A248E76}">
   <dimension ref="A1:Y183"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="11" max="11" width="19" customWidth="1"/>
-    <col min="20" max="20" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="29.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="4" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4661,7 +4661,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -4720,7 +4720,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>79</v>
       </c>
@@ -4791,7 +4791,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -4856,7 +4856,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>79</v>
       </c>
@@ -4921,7 +4921,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -4989,7 +4989,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -5057,7 +5057,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>79</v>
       </c>
@@ -5125,7 +5125,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>79</v>
       </c>
@@ -5193,7 +5193,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>79</v>
       </c>
@@ -5261,7 +5261,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -5329,7 +5329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>79</v>
       </c>
@@ -5397,7 +5397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>79</v>
       </c>
@@ -5465,7 +5465,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>79</v>
       </c>
@@ -5533,7 +5533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>79</v>
       </c>
@@ -5598,7 +5598,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -5654,7 +5654,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -5722,7 +5722,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>79</v>
       </c>
@@ -5775,7 +5775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>79</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>79</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>0.997</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>79</v>
       </c>
@@ -5959,7 +5959,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>79</v>
       </c>
@@ -6019,7 +6019,7 @@
         <v>1.0009999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>79</v>
       </c>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="V23" s="8"/>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>79</v>
       </c>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="V24" s="8"/>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -6198,7 +6198,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -6251,7 +6251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>79</v>
       </c>
@@ -6304,7 +6304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -6410,7 +6410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>79</v>
       </c>
@@ -6463,7 +6463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>79</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>79</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>79</v>
       </c>
@@ -6622,7 +6622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>79</v>
       </c>
@@ -6675,7 +6675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>79</v>
       </c>
@@ -6728,7 +6728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>79</v>
       </c>
@@ -6781,7 +6781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -6834,7 +6834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>79</v>
       </c>
@@ -6887,7 +6887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>79</v>
       </c>
@@ -6940,7 +6940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -6993,7 +6993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>79</v>
       </c>
@@ -7046,7 +7046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -7099,7 +7099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>79</v>
       </c>
@@ -7152,7 +7152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>79</v>
       </c>
@@ -7205,7 +7205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>79</v>
       </c>
@@ -7261,7 +7261,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>79</v>
       </c>
@@ -7314,7 +7314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>79</v>
       </c>
@@ -7367,7 +7367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>79</v>
       </c>
@@ -7420,7 +7420,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>79</v>
       </c>
@@ -7473,7 +7473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>79</v>
       </c>
@@ -7526,7 +7526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>79</v>
       </c>
@@ -7579,7 +7579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>79</v>
       </c>
@@ -7632,7 +7632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>79</v>
       </c>
@@ -7685,7 +7685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>79</v>
       </c>
@@ -7738,7 +7738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>79</v>
       </c>
@@ -7791,7 +7791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>79</v>
       </c>
@@ -7844,7 +7844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>79</v>
       </c>
@@ -7897,7 +7897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>79</v>
       </c>
@@ -7950,7 +7950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>79</v>
       </c>
@@ -8003,7 +8003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>79</v>
       </c>
@@ -8056,7 +8056,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>79</v>
       </c>
@@ -8109,7 +8109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>79</v>
       </c>
@@ -8162,7 +8162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>79</v>
       </c>
@@ -8215,7 +8215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>79</v>
       </c>
@@ -8268,7 +8268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>79</v>
       </c>
@@ -8321,7 +8321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>79</v>
       </c>
@@ -8374,7 +8374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>79</v>
       </c>
@@ -8427,7 +8427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>79</v>
       </c>
@@ -8480,7 +8480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -8533,7 +8533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -8586,7 +8586,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>79</v>
       </c>
@@ -8639,7 +8639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>79</v>
       </c>
@@ -8692,7 +8692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>79</v>
       </c>
@@ -8745,7 +8745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>79</v>
       </c>
@@ -8798,7 +8798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>79</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>79</v>
       </c>
@@ -8957,7 +8957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>79</v>
       </c>
@@ -9010,7 +9010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>79</v>
       </c>
@@ -9063,7 +9063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>79</v>
       </c>
@@ -9116,7 +9116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>79</v>
       </c>
@@ -9169,7 +9169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>79</v>
       </c>
@@ -9222,7 +9222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>79</v>
       </c>
@@ -9275,7 +9275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>79</v>
       </c>
@@ -9328,7 +9328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -9381,7 +9381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>79</v>
       </c>
@@ -9434,7 +9434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>79</v>
       </c>
@@ -9487,7 +9487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>79</v>
       </c>
@@ -9540,7 +9540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>79</v>
       </c>
@@ -9593,7 +9593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>79</v>
       </c>
@@ -9646,7 +9646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>79</v>
       </c>
@@ -9699,7 +9699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>79</v>
       </c>
@@ -9752,7 +9752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>79</v>
       </c>
@@ -9805,7 +9805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>79</v>
       </c>
@@ -9858,7 +9858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>79</v>
       </c>
@@ -9911,7 +9911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>79</v>
       </c>
@@ -9964,7 +9964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>79</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>79</v>
       </c>
@@ -10070,7 +10070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>79</v>
       </c>
@@ -10123,7 +10123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>79</v>
       </c>
@@ -10176,7 +10176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>79</v>
       </c>
@@ -10229,7 +10229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>79</v>
       </c>
@@ -10282,7 +10282,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>79</v>
       </c>
@@ -10335,7 +10335,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>79</v>
       </c>
@@ -10388,7 +10388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>79</v>
       </c>
@@ -10441,7 +10441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>79</v>
       </c>
@@ -10494,7 +10494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>79</v>
       </c>
@@ -10535,7 +10535,7 @@
         <v>31</v>
       </c>
       <c r="N107" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="O107">
         <v>1.343</v>
@@ -10547,7 +10547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>79</v>
       </c>
@@ -10600,7 +10600,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>79</v>
       </c>
@@ -10653,7 +10653,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>79</v>
       </c>
@@ -10706,7 +10706,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>79</v>
       </c>
@@ -10759,7 +10759,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>79</v>
       </c>
@@ -10812,7 +10812,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>79</v>
       </c>
@@ -10865,7 +10865,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>79</v>
       </c>
@@ -10918,7 +10918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>79</v>
       </c>
@@ -10971,7 +10971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>79</v>
       </c>
@@ -11024,7 +11024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>79</v>
       </c>
@@ -11077,7 +11077,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>79</v>
       </c>
@@ -11130,7 +11130,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>79</v>
       </c>
@@ -11183,7 +11183,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>79</v>
       </c>
@@ -11236,7 +11236,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>79</v>
       </c>
@@ -11289,7 +11289,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>79</v>
       </c>
@@ -11342,7 +11342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>79</v>
       </c>
@@ -11395,7 +11395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>79</v>
       </c>
@@ -11448,7 +11448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>79</v>
       </c>
@@ -11501,7 +11501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>79</v>
       </c>
@@ -11554,7 +11554,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>79</v>
       </c>
@@ -11607,7 +11607,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>79</v>
       </c>
@@ -11660,7 +11660,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>79</v>
       </c>
@@ -11713,7 +11713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>79</v>
       </c>
@@ -11766,7 +11766,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>79</v>
       </c>
@@ -11819,7 +11819,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>79</v>
       </c>
@@ -11872,7 +11872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>79</v>
       </c>
@@ -11925,7 +11925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>79</v>
       </c>
@@ -11978,7 +11978,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>79</v>
       </c>
@@ -12031,7 +12031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>79</v>
       </c>
@@ -12084,7 +12084,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>79</v>
       </c>
@@ -12137,7 +12137,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>79</v>
       </c>
@@ -12190,7 +12190,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>79</v>
       </c>
@@ -12243,7 +12243,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>79</v>
       </c>
@@ -12296,7 +12296,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>79</v>
       </c>
@@ -12349,7 +12349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>79</v>
       </c>
@@ -12402,7 +12402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>79</v>
       </c>
@@ -12455,7 +12455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>79</v>
       </c>
@@ -12508,7 +12508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>79</v>
       </c>
@@ -12561,7 +12561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>79</v>
       </c>
@@ -12614,7 +12614,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>79</v>
       </c>
@@ -12667,7 +12667,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>79</v>
       </c>
@@ -12720,7 +12720,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>79</v>
       </c>
@@ -12773,7 +12773,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>79</v>
       </c>
@@ -12826,7 +12826,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>79</v>
       </c>
@@ -12879,7 +12879,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>79</v>
       </c>
@@ -12932,7 +12932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>79</v>
       </c>
@@ -12985,7 +12985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>79</v>
       </c>
@@ -13038,7 +13038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>79</v>
       </c>
@@ -13091,7 +13091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>79</v>
       </c>
@@ -13144,7 +13144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>79</v>
       </c>
@@ -13197,7 +13197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>79</v>
       </c>
@@ -13250,7 +13250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>79</v>
       </c>
@@ -13303,7 +13303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>79</v>
       </c>
@@ -13356,7 +13356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>79</v>
       </c>
@@ -13409,7 +13409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>79</v>
       </c>
@@ -13462,7 +13462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>79</v>
       </c>
@@ -13515,7 +13515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>79</v>
       </c>
@@ -13568,7 +13568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>79</v>
       </c>
@@ -13621,7 +13621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>79</v>
       </c>
@@ -13674,7 +13674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>79</v>
       </c>
@@ -13727,7 +13727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>79</v>
       </c>
@@ -13780,7 +13780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>79</v>
       </c>
@@ -13833,7 +13833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>79</v>
       </c>
@@ -13886,7 +13886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>79</v>
       </c>
@@ -13939,7 +13939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>79</v>
       </c>
@@ -13992,7 +13992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>79</v>
       </c>
@@ -14045,7 +14045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>79</v>
       </c>
@@ -14098,7 +14098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>79</v>
       </c>
@@ -14151,7 +14151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A176" s="6" t="s">
         <v>79</v>
       </c>
@@ -14204,7 +14204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
         <v>79</v>
       </c>
@@ -14257,7 +14257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>79</v>
       </c>
@@ -14310,7 +14310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>79</v>
       </c>
@@ -14363,7 +14363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A180" s="6" t="s">
         <v>79</v>
       </c>
@@ -14404,7 +14404,7 @@
         <v>31</v>
       </c>
       <c r="N180" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="O180" s="6" t="s">
         <v>36</v>
@@ -14416,7 +14416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A181" s="6" t="s">
         <v>79</v>
       </c>
@@ -14457,7 +14457,7 @@
         <v>31</v>
       </c>
       <c r="N181" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="O181" s="6" t="s">
         <v>36</v>
@@ -14469,7 +14469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A182" s="6" t="s">
         <v>79</v>
       </c>
@@ -14522,7 +14522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
         <v>79</v>
       </c>

</xml_diff>

<commit_message>
update to several raw data files - updated in box
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/Erie/D100/ER 10 D100 Spring 2024 24GE00I73 Zoop.xlsx
+++ b/data/raw/GLNPO 2024 Spring/Erie/D100/ER 10 D100 Spring 2024 24GE00I73 Zoop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\Erie\D100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7799DF54-DF35-4256-9F4D-2BD4CFAD0DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B283D4A-10E8-48E4-8DB2-FAB5843CDD56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{80FB5747-2496-44F2-ACA5-DE03CA5C5388}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId2"/>
+    <pivotCache cacheId="31" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -4146,7 +4146,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{75DDA9CE-6863-4D74-9189-5E1074C0BE29}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{75DDA9CE-6863-4D74-9189-5E1074C0BE29}" name="PivotTable1" cacheId="31" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="T2:Y17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
@@ -4593,6 +4593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A2BCB1-26C9-4765-B0C9-78158A248E76}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:Y183"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4720,7 +4721,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>79</v>
       </c>
@@ -4791,7 +4792,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -4856,7 +4857,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>79</v>
       </c>
@@ -4921,7 +4922,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>79</v>
       </c>
@@ -4989,7 +4990,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -5125,7 +5126,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>79</v>
       </c>
@@ -5193,7 +5194,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>79</v>
       </c>
@@ -5261,7 +5262,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>79</v>
       </c>
@@ -5329,7 +5330,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>79</v>
       </c>
@@ -5397,7 +5398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>79</v>
       </c>
@@ -5465,7 +5466,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>79</v>
       </c>
@@ -5533,7 +5534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>79</v>
       </c>
@@ -5598,7 +5599,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>79</v>
       </c>
@@ -5654,7 +5655,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -5775,7 +5776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>79</v>
       </c>
@@ -5837,7 +5838,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>79</v>
       </c>
@@ -5897,7 +5898,7 @@
         <v>0.997</v>
       </c>
     </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>79</v>
       </c>
@@ -5959,7 +5960,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>79</v>
       </c>
@@ -6019,7 +6020,7 @@
         <v>1.0009999999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>79</v>
       </c>
@@ -6079,7 +6080,7 @@
       </c>
       <c r="V23" s="8"/>
     </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>79</v>
       </c>
@@ -6139,7 +6140,7 @@
       </c>
       <c r="V24" s="8"/>
     </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -6198,7 +6199,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -6251,7 +6252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>79</v>
       </c>
@@ -6304,7 +6305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -6357,7 +6358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -6410,7 +6411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>79</v>
       </c>
@@ -6516,7 +6517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:25" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>79</v>
       </c>
@@ -6569,7 +6570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>79</v>
       </c>
@@ -6622,7 +6623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>79</v>
       </c>
@@ -6728,7 +6729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>79</v>
       </c>
@@ -6781,7 +6782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -6887,7 +6888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>79</v>
       </c>
@@ -6940,7 +6941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -6993,7 +6994,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>79</v>
       </c>
@@ -7099,7 +7100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>79</v>
       </c>
@@ -7261,7 +7262,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>79</v>
       </c>
@@ -7314,7 +7315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>79</v>
       </c>
@@ -7367,7 +7368,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:18" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>79</v>
       </c>
@@ -7420,7 +7421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>79</v>
       </c>
@@ -7473,7 +7474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>79</v>
       </c>
@@ -7579,7 +7580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>79</v>
       </c>
@@ -7632,7 +7633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>79</v>
       </c>
@@ -7685,7 +7686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>79</v>
       </c>
@@ -7738,7 +7739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>79</v>
       </c>
@@ -7791,7 +7792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>79</v>
       </c>
@@ -7844,7 +7845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>79</v>
       </c>
@@ -7897,7 +7898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>79</v>
       </c>
@@ -7950,7 +7951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>79</v>
       </c>
@@ -8003,7 +8004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>79</v>
       </c>
@@ -8056,7 +8057,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>79</v>
       </c>
@@ -8109,7 +8110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>79</v>
       </c>
@@ -8162,7 +8163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>79</v>
       </c>
@@ -8215,7 +8216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>79</v>
       </c>
@@ -8268,7 +8269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>79</v>
       </c>
@@ -8321,7 +8322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>79</v>
       </c>
@@ -8374,7 +8375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>79</v>
       </c>
@@ -8480,7 +8481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -8533,7 +8534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -8586,7 +8587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>79</v>
       </c>
@@ -8639,7 +8640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>79</v>
       </c>
@@ -8745,7 +8746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>79</v>
       </c>
@@ -8798,7 +8799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>79</v>
       </c>
@@ -8851,7 +8852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -9010,7 +9011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>79</v>
       </c>
@@ -9116,7 +9117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>79</v>
       </c>
@@ -9169,7 +9170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>79</v>
       </c>
@@ -9328,7 +9329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>79</v>
       </c>
@@ -9381,7 +9382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>79</v>
       </c>
@@ -9540,7 +9541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>79</v>
       </c>
@@ -9593,7 +9594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>79</v>
       </c>
@@ -9646,7 +9647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>79</v>
       </c>
@@ -9699,7 +9700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>79</v>
       </c>
@@ -9752,7 +9753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>79</v>
       </c>
@@ -9805,7 +9806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>79</v>
       </c>
@@ -9858,7 +9859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>79</v>
       </c>
@@ -10017,7 +10018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>79</v>
       </c>
@@ -10070,7 +10071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>79</v>
       </c>
@@ -10123,7 +10124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>79</v>
       </c>
@@ -10176,7 +10177,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>79</v>
       </c>
@@ -10229,7 +10230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>79</v>
       </c>
@@ -10282,7 +10283,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>79</v>
       </c>
@@ -10335,7 +10336,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>79</v>
       </c>
@@ -10388,7 +10389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>79</v>
       </c>
@@ -10441,7 +10442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>79</v>
       </c>
@@ -10494,7 +10495,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>79</v>
       </c>
@@ -10653,7 +10654,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>79</v>
       </c>
@@ -10706,7 +10707,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>79</v>
       </c>
@@ -10759,7 +10760,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>79</v>
       </c>
@@ -10812,7 +10813,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>79</v>
       </c>
@@ -10865,7 +10866,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>79</v>
       </c>
@@ -10918,7 +10919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>79</v>
       </c>
@@ -10971,7 +10972,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>79</v>
       </c>
@@ -11130,7 +11131,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>79</v>
       </c>
@@ -11183,7 +11184,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>79</v>
       </c>
@@ -11236,7 +11237,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>79</v>
       </c>
@@ -11289,7 +11290,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>79</v>
       </c>
@@ -11342,7 +11343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>79</v>
       </c>
@@ -11395,7 +11396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>79</v>
       </c>
@@ -11448,7 +11449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>79</v>
       </c>
@@ -11601,13 +11602,13 @@
         <v>36</v>
       </c>
       <c r="P127" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="Q127">
         <v>5</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>79</v>
       </c>
@@ -11660,7 +11661,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>79</v>
       </c>
@@ -11713,7 +11714,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>79</v>
       </c>
@@ -11766,7 +11767,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>79</v>
       </c>
@@ -11819,7 +11820,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>79</v>
       </c>
@@ -11872,7 +11873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>79</v>
       </c>
@@ -12031,7 +12032,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>79</v>
       </c>
@@ -12084,7 +12085,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>79</v>
       </c>
@@ -12137,7 +12138,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>79</v>
       </c>
@@ -12190,7 +12191,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>79</v>
       </c>
@@ -12243,7 +12244,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>79</v>
       </c>
@@ -12296,7 +12297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>79</v>
       </c>
@@ -12349,7 +12350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>79</v>
       </c>
@@ -12402,7 +12403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>79</v>
       </c>
@@ -12455,7 +12456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>79</v>
       </c>
@@ -12508,7 +12509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>79</v>
       </c>
@@ -12667,7 +12668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>79</v>
       </c>
@@ -12720,7 +12721,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>79</v>
       </c>
@@ -12773,7 +12774,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>79</v>
       </c>
@@ -12826,7 +12827,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>79</v>
       </c>
@@ -12879,7 +12880,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>79</v>
       </c>
@@ -12932,7 +12933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>79</v>
       </c>
@@ -12985,7 +12986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>79</v>
       </c>
@@ -13038,7 +13039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>79</v>
       </c>
@@ -13091,7 +13092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>79</v>
       </c>
@@ -13144,7 +13145,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>79</v>
       </c>
@@ -13197,7 +13198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>79</v>
       </c>
@@ -13250,7 +13251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>79</v>
       </c>
@@ -13303,7 +13304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>79</v>
       </c>
@@ -13356,7 +13357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>79</v>
       </c>
@@ -13409,7 +13410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>79</v>
       </c>
@@ -13462,7 +13463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>79</v>
       </c>
@@ -13515,7 +13516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>79</v>
       </c>
@@ -13568,7 +13569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>79</v>
       </c>
@@ -13621,7 +13622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>79</v>
       </c>
@@ -13674,7 +13675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>79</v>
       </c>
@@ -13727,7 +13728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>79</v>
       </c>
@@ -13780,7 +13781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>79</v>
       </c>
@@ -13833,7 +13834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>79</v>
       </c>
@@ -13886,7 +13887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>79</v>
       </c>
@@ -13939,7 +13940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>79</v>
       </c>
@@ -13992,7 +13993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>79</v>
       </c>
@@ -14045,7 +14046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>79</v>
       </c>
@@ -14098,7 +14099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>79</v>
       </c>
@@ -14151,7 +14152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="6" t="s">
         <v>79</v>
       </c>
@@ -14204,7 +14205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
         <v>79</v>
       </c>
@@ -14257,7 +14258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>79</v>
       </c>
@@ -14310,7 +14311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>79</v>
       </c>
@@ -14363,7 +14364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="6" t="s">
         <v>79</v>
       </c>
@@ -14416,7 +14417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="6" t="s">
         <v>79</v>
       </c>
@@ -14469,7 +14470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="6" t="s">
         <v>79</v>
       </c>
@@ -14522,7 +14523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:17" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="6" t="s">
         <v>79</v>
       </c>
@@ -14576,6 +14577,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:R183" xr:uid="{45A2BCB1-26C9-4765-B0C9-78158A248E76}">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="Diacyclops thomasi"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>